<commit_message>
new save, only a field name changed
</commit_message>
<xml_diff>
--- a/input/input_cal_PR.xlsx
+++ b/input/input_cal_PR.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="343" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12B68E4D-E8A8-4F7C-AEC7-BD8D134FAA8E}"/>
+  <xr:revisionPtr revIDLastSave="447" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{163659DD-EFFC-48EA-9CB7-851F6A4AE764}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="22">
   <si>
     <t>Fluid</t>
   </si>
@@ -94,15 +93,25 @@
   </si>
   <si>
     <t>H275CO2</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>Mpa</t>
+  </si>
+  <si>
+    <t>CH4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00000"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -145,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -159,7 +168,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -442,16 +454,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="8.85546875" style="2"/>
-    <col min="5" max="5" width="7.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="11.28515625" style="2" customWidth="1"/>
+    <col min="5" max="6" width="7.42578125" style="2" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -468,13 +480,19 @@
         <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
@@ -487,11 +505,14 @@
       <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -510,13 +531,20 @@
         <v>1.0135649999999998</v>
       </c>
       <c r="F3" s="5">
+        <f>E3*0.1</f>
+        <v>0.10135649999999999</v>
+      </c>
+      <c r="G3" s="6">
         <v>7.9399999999999998E-2</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="6">
+        <v>1.0003</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -535,13 +563,20 @@
         <v>4.4610649999999996</v>
       </c>
       <c r="F4" s="5">
+        <f t="shared" ref="F4:F37" si="2">E4*0.1</f>
+        <v>0.44610649999999996</v>
+      </c>
+      <c r="G4" s="6">
         <v>0.3175</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="6">
+        <v>1.0011000000000001</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -560,13 +595,20 @@
         <v>14.803564999999999</v>
       </c>
       <c r="F5" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4803565000000001</v>
+      </c>
+      <c r="G5" s="6">
         <v>1.1868000000000001</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="6">
+        <v>1.0043</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
@@ -585,13 +627,20 @@
         <v>35.488565000000001</v>
       </c>
       <c r="F6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.5488565000000003</v>
+      </c>
+      <c r="G6" s="6">
         <v>2.7519999999999998</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="6">
+        <v>1.0105999999999999</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -610,13 +659,20 @@
         <v>63.068565</v>
       </c>
       <c r="F7" s="5">
+        <f t="shared" si="2"/>
+        <v>6.3068565000000003</v>
+      </c>
+      <c r="G7" s="6">
         <v>4.9062000000000001</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="6">
+        <v>1.0204</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -635,13 +691,20 @@
         <v>104.438565</v>
       </c>
       <c r="F8" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443856500000001</v>
+      </c>
+      <c r="G8" s="6">
         <v>7.9736000000000002</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="6">
+        <v>1.0364</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -660,13 +723,20 @@
         <v>1.0135649999999998</v>
       </c>
       <c r="F9" s="5">
+        <f t="shared" si="2"/>
+        <v>0.10135649999999999</v>
+      </c>
+      <c r="G9" s="6">
         <v>0.15759999999999999</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="6">
+        <v>1.0002</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -685,13 +755,20 @@
         <v>4.4610649999999996</v>
       </c>
       <c r="F10" s="5">
+        <f t="shared" si="2"/>
+        <v>0.44610649999999996</v>
+      </c>
+      <c r="G10" s="6">
         <v>0.63029999999999997</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="6">
+        <v>1.0005999999999999</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -710,13 +787,20 @@
         <v>14.803564999999999</v>
       </c>
       <c r="F11" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4803565000000001</v>
+      </c>
+      <c r="G11" s="6">
         <v>2.3591000000000002</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="6">
+        <v>1.0024999999999999</v>
+      </c>
+      <c r="I11" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -735,13 +819,20 @@
         <v>35.488565000000001</v>
       </c>
       <c r="F12" s="5">
+        <f t="shared" si="2"/>
+        <v>3.5488565000000003</v>
+      </c>
+      <c r="G12" s="6">
         <v>5.4836</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="6">
+        <v>1.0063</v>
+      </c>
+      <c r="I12" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
@@ -760,13 +851,20 @@
         <v>63.068565</v>
       </c>
       <c r="F13" s="5">
+        <f t="shared" si="2"/>
+        <v>6.3068565000000003</v>
+      </c>
+      <c r="G13" s="6">
         <v>9.8087</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="H13" s="6">
+        <v>1.0126999999999999</v>
+      </c>
+      <c r="I13" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -785,13 +883,20 @@
         <v>104.438565</v>
       </c>
       <c r="F14" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443856500000001</v>
+      </c>
+      <c r="G14" s="6">
         <v>16.0169</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="H14" s="6">
+        <v>1.0237000000000001</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -810,13 +915,20 @@
         <v>1.0135649999999998</v>
       </c>
       <c r="F15" s="5">
+        <f t="shared" si="2"/>
+        <v>0.10135649999999999</v>
+      </c>
+      <c r="G15" s="6">
         <v>1.7436</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="H15" s="6">
+        <v>0.99490000000000001</v>
+      </c>
+      <c r="I15" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>11</v>
       </c>
@@ -835,13 +947,20 @@
         <v>4.4610649999999996</v>
       </c>
       <c r="F16" s="5">
+        <f t="shared" si="2"/>
+        <v>0.44610649999999996</v>
+      </c>
+      <c r="G16" s="6">
         <v>7.0845000000000002</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="H16" s="6">
+        <v>0.97940000000000005</v>
+      </c>
+      <c r="I16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
@@ -860,13 +979,20 @@
         <v>14.803564999999999</v>
       </c>
       <c r="F17" s="5">
+        <f t="shared" si="2"/>
+        <v>1.4803565000000001</v>
+      </c>
+      <c r="G17" s="6">
         <v>28.2637</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="6">
+        <v>0.92059999999999997</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>11</v>
       </c>
@@ -885,13 +1011,20 @@
         <v>35.488565000000001</v>
       </c>
       <c r="F18" s="5">
+        <f t="shared" si="2"/>
+        <v>3.5488565000000003</v>
+      </c>
+      <c r="G18" s="6">
         <v>75.694199999999995</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="H18" s="6">
+        <v>0.80210000000000004</v>
+      </c>
+      <c r="I18" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>11</v>
       </c>
@@ -910,13 +1043,20 @@
         <v>63.068565</v>
       </c>
       <c r="F19" s="5">
+        <f t="shared" si="2"/>
+        <v>6.3068565000000003</v>
+      </c>
+      <c r="G19" s="6">
         <v>188.47470000000001</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="6">
+        <v>0.57979999999999998</v>
+      </c>
+      <c r="I19" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>11</v>
       </c>
@@ -935,13 +1075,20 @@
         <v>104.438565</v>
       </c>
       <c r="F20" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443856500000001</v>
+      </c>
+      <c r="G20" s="6">
         <v>709.51559999999995</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="H20" s="6">
+        <v>0.25430000000000003</v>
+      </c>
+      <c r="I20" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
@@ -960,13 +1107,20 @@
         <v>104.438565</v>
       </c>
       <c r="F21" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443856500000001</v>
+      </c>
+      <c r="G21" s="6">
         <v>117.5121</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="6">
+        <v>0.99019999999999997</v>
+      </c>
+      <c r="I21" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>16</v>
       </c>
@@ -977,21 +1131,28 @@
         <v>116</v>
       </c>
       <c r="D22" s="2">
-        <f t="shared" ref="D22:D27" si="2">C22+14.7</f>
+        <f t="shared" ref="D22:D27" si="3">C22+14.7</f>
         <v>130.69999999999999</v>
       </c>
       <c r="E22" s="4">
-        <f t="shared" ref="E22:E27" si="3">D22/14.5038</f>
+        <f t="shared" ref="E22:E27" si="4">D22/14.5038</f>
         <v>9.0114314869206691</v>
       </c>
       <c r="F22" s="5">
+        <f t="shared" si="2"/>
+        <v>0.90114314869206691</v>
+      </c>
+      <c r="G22" s="6">
         <v>49.884999999999998</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="6">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>16</v>
       </c>
@@ -1002,21 +1163,28 @@
         <v>246</v>
       </c>
       <c r="D23" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>260.7</v>
       </c>
       <c r="E23" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>17.97459976006288</v>
       </c>
       <c r="F23" s="5">
+        <f t="shared" si="2"/>
+        <v>1.7974599760062882</v>
+      </c>
+      <c r="G23" s="6">
         <v>106.1506</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="6">
+        <v>0.88919999999999999</v>
+      </c>
+      <c r="I23" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>16</v>
       </c>
@@ -1027,21 +1195,28 @@
         <v>348</v>
       </c>
       <c r="D24" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>362.7</v>
       </c>
       <c r="E24" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25.007239482066769</v>
       </c>
-      <c r="F24" s="2">
+      <c r="F24" s="5">
+        <f t="shared" si="2"/>
+        <v>2.500723948206677</v>
+      </c>
+      <c r="G24" s="6">
         <v>155.6155</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="H24" s="6">
+        <v>0.84240000000000004</v>
+      </c>
+      <c r="I24" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -1052,21 +1227,28 @@
         <v>450</v>
       </c>
       <c r="D25" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>464.7</v>
       </c>
       <c r="E25" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>32.039879204070658</v>
       </c>
-      <c r="F25" s="2">
+      <c r="F25" s="5">
+        <f t="shared" si="2"/>
+        <v>3.2039879204070658</v>
+      </c>
+      <c r="G25" s="6">
         <v>211.64850000000001</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="H25" s="6">
+        <v>0.79279999999999995</v>
+      </c>
+      <c r="I25" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>16</v>
       </c>
@@ -1077,21 +1259,28 @@
         <v>550</v>
       </c>
       <c r="D26" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>564.70000000000005</v>
       </c>
       <c r="E26" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>38.934624029564667</v>
       </c>
-      <c r="F26" s="2">
+      <c r="F26" s="5">
+        <f t="shared" si="2"/>
+        <v>3.8934624029564668</v>
+      </c>
+      <c r="G26" s="6">
         <v>276.53210000000001</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="H26" s="6">
+        <v>0.73950000000000005</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>16</v>
       </c>
@@ -1102,21 +1291,28 @@
         <v>650</v>
       </c>
       <c r="D27" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>664.7</v>
       </c>
       <c r="E27" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>45.829368855058675</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="5">
+        <f t="shared" si="2"/>
+        <v>4.5829368855058679</v>
+      </c>
+      <c r="G27" s="6">
         <v>354.10019999999997</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="H27" s="6">
+        <v>0.68120000000000003</v>
+      </c>
+      <c r="I27" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>16</v>
       </c>
@@ -1127,21 +1323,28 @@
         <v>725</v>
       </c>
       <c r="D28" s="2">
-        <f t="shared" ref="D28:D35" si="4">C28+14.7</f>
+        <f t="shared" ref="D28:D40" si="5">C28+14.7</f>
         <v>739.7</v>
       </c>
       <c r="E28" s="4">
-        <f t="shared" ref="E28:E35" si="5">D28/14.5038</f>
+        <f t="shared" ref="E28:E40" si="6">D28/14.5038</f>
         <v>51.000427474179183</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F28" s="5">
+        <f t="shared" si="2"/>
+        <v>5.1000427474179189</v>
+      </c>
+      <c r="G28" s="6">
         <v>421.04160000000002</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="H28" s="6">
+        <v>0.63519999999999999</v>
+      </c>
+      <c r="I28" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>16</v>
       </c>
@@ -1152,21 +1355,28 @@
         <v>900</v>
       </c>
       <c r="D29" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>914.7</v>
       </c>
       <c r="E29" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>63.0662309187937</v>
       </c>
-      <c r="F29" s="2">
+      <c r="F29" s="5">
+        <f t="shared" si="2"/>
+        <v>6.30662309187937</v>
+      </c>
+      <c r="G29" s="6">
         <v>664.28779999999995</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="H29" s="6">
+        <v>0.49730000000000002</v>
+      </c>
+      <c r="I29" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>17</v>
       </c>
@@ -1177,18 +1387,25 @@
         <v>1500</v>
       </c>
       <c r="D30" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1514.7</v>
       </c>
-      <c r="E30" s="2">
-        <f t="shared" si="5"/>
+      <c r="E30" s="4">
+        <f t="shared" si="6"/>
         <v>104.43469987175774</v>
       </c>
       <c r="F30" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443469987175774</v>
+      </c>
+      <c r="G30" s="6">
         <v>108.68918417822</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30" s="6">
+        <v>0.87949999999999995</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>18</v>
       </c>
@@ -1199,70 +1416,85 @@
         <v>1500</v>
       </c>
       <c r="D31" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1514.7</v>
       </c>
-      <c r="E31" s="2">
-        <f t="shared" si="5"/>
+      <c r="E31" s="4">
+        <f t="shared" si="6"/>
         <v>104.43469987175774</v>
       </c>
-      <c r="F31" s="2">
+      <c r="F31" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443469987175774</v>
+      </c>
+      <c r="G31" s="6">
         <v>52.7830901560271</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" s="6">
+        <v>0.98480000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="2">
+        <v>32</v>
+      </c>
+      <c r="C32" s="2">
+        <v>1500</v>
+      </c>
+      <c r="D32" s="2">
+        <f t="shared" ref="D32:D33" si="7">C32+14.7</f>
+        <v>1514.7</v>
+      </c>
+      <c r="E32" s="4">
+        <f t="shared" ref="E32:E33" si="8">D32/14.5038</f>
+        <v>104.43469987175774</v>
+      </c>
+      <c r="F32" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443469987175774</v>
+      </c>
+      <c r="G32" s="6">
+        <v>106.43810000000001</v>
+      </c>
+      <c r="H32" s="6">
+        <v>0.88629999999999998</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="2">
+        <v>32</v>
+      </c>
+      <c r="C33" s="2">
+        <v>1500</v>
+      </c>
+      <c r="D33" s="2">
+        <f t="shared" si="7"/>
+        <v>1514.7</v>
+      </c>
+      <c r="E33" s="4">
+        <f t="shared" si="8"/>
+        <v>104.43469987175774</v>
+      </c>
+      <c r="F33" s="5">
+        <f t="shared" si="2"/>
+        <v>10.443469987175774</v>
+      </c>
+      <c r="G33" s="6">
+        <v>51.974600000000002</v>
+      </c>
+      <c r="H33" s="6">
+        <v>0.98699999999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B32" s="2">
-        <v>20</v>
-      </c>
-      <c r="C32" s="2">
-        <v>725</v>
-      </c>
-      <c r="D32" s="2">
-        <f t="shared" si="4"/>
-        <v>739.7</v>
-      </c>
-      <c r="E32" s="2">
-        <f t="shared" si="5"/>
-        <v>51.000427474179183</v>
-      </c>
-      <c r="F32" s="2">
-        <v>8.2866999999999997</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33" s="2">
-        <v>20</v>
-      </c>
-      <c r="C33" s="2">
-        <v>900</v>
-      </c>
-      <c r="D33" s="2">
-        <f t="shared" si="4"/>
-        <v>914.7</v>
-      </c>
-      <c r="E33" s="2">
-        <f t="shared" si="5"/>
-        <v>63.0662309187937</v>
-      </c>
-      <c r="F33" s="2">
-        <v>10.2066</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="B34" s="2">
         <v>20</v>
@@ -1271,23 +1503,30 @@
         <v>725</v>
       </c>
       <c r="D34" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>739.7</v>
       </c>
-      <c r="E34" s="2">
-        <f t="shared" si="5"/>
+      <c r="E34" s="4">
+        <f t="shared" si="6"/>
         <v>51.000427474179183</v>
       </c>
-      <c r="F34" s="2">
-        <v>471.17140000000001</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F34" s="5">
+        <f t="shared" si="2"/>
+        <v>5.1000427474179189</v>
+      </c>
+      <c r="G34" s="6">
+        <v>8.2866999999999997</v>
+      </c>
+      <c r="H34" s="6">
+        <v>1.0101</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B35" s="2">
         <v>20</v>
@@ -1296,17 +1535,184 @@
         <v>900</v>
       </c>
       <c r="D35" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>914.7</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35" s="4">
+        <f t="shared" si="6"/>
+        <v>63.0662309187937</v>
+      </c>
+      <c r="F35" s="5">
+        <f t="shared" si="2"/>
+        <v>6.30662309187937</v>
+      </c>
+      <c r="G35" s="6">
+        <v>10.2066</v>
+      </c>
+      <c r="H35" s="6">
+        <v>1.0129999999999999</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" s="2">
+        <v>20</v>
+      </c>
+      <c r="C36" s="2">
+        <v>725</v>
+      </c>
+      <c r="D36" s="2">
         <f t="shared" si="5"/>
+        <v>739.7</v>
+      </c>
+      <c r="E36" s="4">
+        <f t="shared" si="6"/>
+        <v>51.000427474179183</v>
+      </c>
+      <c r="F36" s="5">
+        <f t="shared" si="2"/>
+        <v>5.1000427474179189</v>
+      </c>
+      <c r="G36" s="6">
+        <v>471.17140000000001</v>
+      </c>
+      <c r="H36" s="6">
+        <v>0.58309999999999995</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="2">
+        <v>20</v>
+      </c>
+      <c r="C37" s="2">
+        <v>900</v>
+      </c>
+      <c r="D37" s="2">
+        <f t="shared" si="5"/>
+        <v>914.7</v>
+      </c>
+      <c r="E37" s="4">
+        <f t="shared" si="6"/>
         <v>63.0662309187937</v>
       </c>
-      <c r="F35" s="2">
+      <c r="F37" s="5">
+        <f t="shared" si="2"/>
+        <v>6.30662309187937</v>
+      </c>
+      <c r="G37" s="6">
         <v>1148.7</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="H37" s="6">
+        <v>0.2954</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="2">
+        <v>40</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1160</v>
+      </c>
+      <c r="D38" s="2">
+        <f t="shared" si="5"/>
+        <v>1174.7</v>
+      </c>
+      <c r="E38" s="4">
+        <f t="shared" si="6"/>
+        <v>80.992567465078125</v>
+      </c>
+      <c r="F38" s="5">
+        <f>E38*0.1</f>
+        <v>8.0992567465078125</v>
+      </c>
+      <c r="G38" s="2">
+        <v>295.86799999999999</v>
+      </c>
+      <c r="H38" s="2">
+        <v>0.46339999999999998</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" s="2">
+        <v>40</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1160</v>
+      </c>
+      <c r="D39" s="2">
+        <f t="shared" si="5"/>
+        <v>1174.7</v>
+      </c>
+      <c r="E39" s="4">
+        <f t="shared" si="6"/>
+        <v>80.992567465078125</v>
+      </c>
+      <c r="F39" s="5">
+        <f t="shared" ref="F39:F40" si="9">E39*0.1</f>
+        <v>8.0992567465078125</v>
+      </c>
+      <c r="G39" s="6">
+        <v>87.733400000000003</v>
+      </c>
+      <c r="H39" s="6">
+        <v>0.99339999999999995</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B40" s="2">
+        <v>40</v>
+      </c>
+      <c r="C40" s="2">
+        <v>1160</v>
+      </c>
+      <c r="D40" s="2">
+        <f t="shared" si="5"/>
+        <v>1174.7</v>
+      </c>
+      <c r="E40" s="4">
+        <f t="shared" si="6"/>
+        <v>80.992567465078125</v>
+      </c>
+      <c r="F40" s="5">
+        <f t="shared" si="9"/>
+        <v>8.0992567465078125</v>
+      </c>
+      <c r="G40" s="2">
+        <v>56.8795</v>
+      </c>
+      <c r="H40" s="2">
+        <v>0.87729999999999997</v>
+      </c>
+      <c r="I40" s="4" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
input cal now takes only full cal exp data, that means, one fluid, one temp ref, many P many Q. Input fields were changed to capture that and also capture pump working for each experiment. Sya Pworking, Pcushion, P confining. This will be transalated to import in data of the BT exps too.
The cal data is now references for each T_MFM using PR EOS for an array of temperatures for each fluid and P and x, and then interpolates for the measured T_MFM
</commit_message>
<xml_diff>
--- a/input/input_cal_PR.xlsx
+++ b/input/input_cal_PR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="447" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{163659DD-EFFC-48EA-9CB7-851F6A4AE764}"/>
+  <xr:revisionPtr revIDLastSave="449" documentId="11_F25DC773A252ABDACC1048B8D1997AFC5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC54A723-51A4-4488-9D07-ABFCAC79CB09}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,8 +110,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -168,10 +168,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -687,11 +687,11 @@
         <v>1514.7</v>
       </c>
       <c r="E8" s="4">
-        <f t="shared" si="1"/>
+        <f>D8*0.06895</f>
         <v>104.438565</v>
       </c>
       <c r="F8" s="5">
-        <f t="shared" si="2"/>
+        <f>E8*0.1</f>
         <v>10.443856500000001</v>
       </c>
       <c r="G8" s="6">

</xml_diff>